<commit_message>
Audit Home financials, rename Milk Sold, refine executive summary
Recalculate COGS, gross margin, total costs, and operating margin for
both TTM windows directly from Monthly Revenue vs. Operating Costs.xlsx
(summed month by month), replacing Key Metrics at a Glance.xlsx's
Operating Margin entry, which didn't reconcile with its own Revenue/
Costs cells and had the YoY direction reversed. Surface the underlying
finding (COGS dropped sharply starting Jan 2026 while total operating
costs barely moved, suggesting a COGS/Expenses reclassification) in the
executive summary rather than presenting the margin gain at face value.

Also: rename "Milk Sold" to "Milk Produced" on the stat card and in
copy, drop Gross Margin from the Key Metrics table per feedback, and
add a footnote clarifying the Net Income stat card includes Other
Income/Expenses (unlike the chart below it, which excludes them).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Monthly Revenue vs. Operating Costs.xlsx
+++ b/data/Monthly Revenue vs. Operating Costs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oliviaarkema/Documents/Strategic Planning/CD_StrategicPlanning/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F88386ED-6295-464D-8C46-94F6C4831637}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC83C91C-6B59-C848-9493-64C92FABA782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3820" yWindow="2320" windowWidth="23720" windowHeight="15040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="-5700" windowWidth="38400" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -33,25 +33,35 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Month</t>
-  </si>
-  <si>
-    <t>Net Income (Including Other Income &amp; Expenses)</t>
   </si>
   <si>
     <t>Revenue $</t>
   </si>
   <si>
-    <t>Costs $ (COGS + Expenses)</t>
+    <t>Operating Costs $ (COGS + Expenses)</t>
+  </si>
+  <si>
+    <t>COGS</t>
+  </si>
+  <si>
+    <t>Expenses</t>
+  </si>
+  <si>
+    <t>Net Ordinary Income (Not Including Other Income &amp; Expenses)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -64,6 +74,13 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -83,15 +100,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Currency" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -392,391 +412,583 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="17" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="2" max="4" width="17" customWidth="1"/>
+    <col min="5" max="5" width="24" customWidth="1"/>
+    <col min="6" max="6" width="13.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="2">
         <v>45474</v>
       </c>
-      <c r="B2">
-        <v>1645545</v>
-      </c>
-      <c r="C2">
-        <f>B2-D2</f>
-        <v>1087512</v>
-      </c>
-      <c r="D2">
-        <v>558033</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B2" s="3">
+        <v>2349438</v>
+      </c>
+      <c r="C2" s="3">
+        <v>741576</v>
+      </c>
+      <c r="D2" s="3">
+        <v>1373637</v>
+      </c>
+      <c r="E2" s="3">
+        <f>C2+D2</f>
+        <v>2115213</v>
+      </c>
+      <c r="F2" s="3">
+        <f>B2-E2</f>
+        <v>234225</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>45505</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="3">
         <v>2299610</v>
       </c>
-      <c r="C3">
-        <f t="shared" ref="C3:C26" si="0">B3-D3</f>
-        <v>2341380</v>
-      </c>
-      <c r="D3">
-        <v>-41770</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C3" s="3">
+        <v>693389</v>
+      </c>
+      <c r="D3" s="3">
+        <v>1620287</v>
+      </c>
+      <c r="E3" s="3">
+        <f t="shared" ref="E3:E26" si="0">C3+D3</f>
+        <v>2313676</v>
+      </c>
+      <c r="F3" s="3">
+        <f t="shared" ref="F3:F26" si="1">B3-E3</f>
+        <v>-14066</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>45536</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="3">
         <v>2055377</v>
       </c>
-      <c r="C4">
-        <f t="shared" si="0"/>
-        <v>2149066</v>
-      </c>
-      <c r="D4">
-        <v>-93689</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C4" s="3">
+        <v>660255</v>
+      </c>
+      <c r="D4" s="3">
+        <v>1448248</v>
+      </c>
+      <c r="E4" s="3">
+        <f t="shared" si="0"/>
+        <v>2108503</v>
+      </c>
+      <c r="F4" s="3">
+        <f t="shared" si="1"/>
+        <v>-53126</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>45566</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="3">
         <v>2225430</v>
       </c>
-      <c r="C5">
-        <f t="shared" si="0"/>
-        <v>2077783</v>
-      </c>
-      <c r="D5">
-        <v>147647</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C5" s="3">
+        <v>669932</v>
+      </c>
+      <c r="D5" s="3">
+        <v>1369023</v>
+      </c>
+      <c r="E5" s="3">
+        <f t="shared" si="0"/>
+        <v>2038955</v>
+      </c>
+      <c r="F5" s="3">
+        <f t="shared" si="1"/>
+        <v>186475</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
         <v>45597</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="3">
         <v>2138141</v>
       </c>
-      <c r="C6">
-        <f t="shared" si="0"/>
-        <v>2130164</v>
-      </c>
-      <c r="D6">
-        <v>7977</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C6" s="3">
+        <v>632241</v>
+      </c>
+      <c r="D6" s="3">
+        <v>1460891</v>
+      </c>
+      <c r="E6" s="3">
+        <f t="shared" si="0"/>
+        <v>2093132</v>
+      </c>
+      <c r="F6" s="3">
+        <f t="shared" si="1"/>
+        <v>45009</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
         <v>45627</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="3">
         <v>2086631</v>
       </c>
-      <c r="C7">
-        <f t="shared" si="0"/>
-        <v>2175007</v>
-      </c>
-      <c r="D7">
-        <v>-88376</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C7" s="3">
+        <v>643073</v>
+      </c>
+      <c r="D7" s="3">
+        <v>1500957</v>
+      </c>
+      <c r="E7" s="3">
+        <f t="shared" si="0"/>
+        <v>2144030</v>
+      </c>
+      <c r="F7" s="3">
+        <f t="shared" si="1"/>
+        <v>-57399</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
         <v>45658</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="3">
         <v>2079507</v>
       </c>
-      <c r="C8">
-        <f t="shared" si="0"/>
-        <v>2150906</v>
-      </c>
-      <c r="D8">
-        <v>-71399</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C8" s="3">
+        <v>666557</v>
+      </c>
+      <c r="D8" s="3">
+        <v>1533414</v>
+      </c>
+      <c r="E8" s="3">
+        <f t="shared" si="0"/>
+        <v>2199971</v>
+      </c>
+      <c r="F8" s="3">
+        <f t="shared" si="1"/>
+        <v>-120464</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
         <v>45689</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="3">
         <v>1772753</v>
       </c>
-      <c r="C9">
-        <f t="shared" si="0"/>
-        <v>1836586</v>
-      </c>
-      <c r="D9">
-        <v>-63833</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C9" s="3">
+        <v>528932</v>
+      </c>
+      <c r="D9" s="3">
+        <v>1279876</v>
+      </c>
+      <c r="E9" s="3">
+        <f t="shared" si="0"/>
+        <v>1808808</v>
+      </c>
+      <c r="F9" s="3">
+        <f t="shared" si="1"/>
+        <v>-36055</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
         <v>45717</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="3">
         <v>2087068</v>
       </c>
-      <c r="C10">
-        <f t="shared" si="0"/>
-        <v>1942402</v>
-      </c>
-      <c r="D10">
-        <v>144666</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C10" s="3">
+        <v>606579</v>
+      </c>
+      <c r="D10" s="3">
+        <v>1406315</v>
+      </c>
+      <c r="E10" s="3">
+        <f t="shared" si="0"/>
+        <v>2012894</v>
+      </c>
+      <c r="F10" s="3">
+        <f t="shared" si="1"/>
+        <v>74174</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
         <v>45748</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="3">
         <v>2184308</v>
       </c>
-      <c r="C11">
-        <f t="shared" si="0"/>
-        <v>2111801</v>
-      </c>
-      <c r="D11">
-        <v>72507</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C11" s="3">
+        <v>600333</v>
+      </c>
+      <c r="D11" s="3">
+        <v>1578487</v>
+      </c>
+      <c r="E11" s="3">
+        <f t="shared" si="0"/>
+        <v>2178820</v>
+      </c>
+      <c r="F11" s="3">
+        <f t="shared" si="1"/>
+        <v>5488</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
         <v>45778</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="3">
         <v>2277922</v>
       </c>
-      <c r="C12">
-        <f t="shared" si="0"/>
-        <v>2241576</v>
-      </c>
-      <c r="D12">
-        <v>36346</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C12" s="3">
+        <v>648707</v>
+      </c>
+      <c r="D12" s="3">
+        <v>1562355</v>
+      </c>
+      <c r="E12" s="3">
+        <f t="shared" si="0"/>
+        <v>2211062</v>
+      </c>
+      <c r="F12" s="3">
+        <f t="shared" si="1"/>
+        <v>66860</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
         <v>45809</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="3">
         <v>2523351</v>
       </c>
-      <c r="C13">
-        <f t="shared" si="0"/>
-        <v>2455781</v>
-      </c>
-      <c r="D13">
-        <v>67570</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C13" s="3">
+        <v>734939</v>
+      </c>
+      <c r="D13" s="3">
+        <v>1696517</v>
+      </c>
+      <c r="E13" s="3">
+        <f t="shared" si="0"/>
+        <v>2431456</v>
+      </c>
+      <c r="F13" s="3">
+        <f t="shared" si="1"/>
+        <v>91895</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
         <v>45839</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="3">
         <v>2585013</v>
       </c>
-      <c r="C14">
-        <f t="shared" si="0"/>
-        <v>2572680</v>
-      </c>
-      <c r="D14">
-        <v>12333</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C14" s="3">
+        <v>690795</v>
+      </c>
+      <c r="D14" s="3">
+        <v>1894587</v>
+      </c>
+      <c r="E14" s="3">
+        <f t="shared" si="0"/>
+        <v>2585382</v>
+      </c>
+      <c r="F14" s="3">
+        <f t="shared" si="1"/>
+        <v>-369</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
         <v>45870</v>
       </c>
-      <c r="B15">
-        <v>2446680</v>
-      </c>
-      <c r="C15">
-        <f t="shared" si="0"/>
-        <v>2319274</v>
-      </c>
-      <c r="D15">
-        <v>127406</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B15" s="3">
+        <v>2466680</v>
+      </c>
+      <c r="C15" s="3">
+        <v>747931</v>
+      </c>
+      <c r="D15" s="3">
+        <v>1555538</v>
+      </c>
+      <c r="E15" s="3">
+        <f t="shared" si="0"/>
+        <v>2303469</v>
+      </c>
+      <c r="F15" s="3">
+        <f t="shared" si="1"/>
+        <v>163211</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
         <v>45901</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="3">
         <v>2244856</v>
       </c>
-      <c r="C16">
-        <f t="shared" si="0"/>
-        <v>2320298</v>
-      </c>
-      <c r="D16">
-        <v>-75442</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C16" s="3">
+        <v>686269</v>
+      </c>
+      <c r="D16" s="3">
+        <v>1617567</v>
+      </c>
+      <c r="E16" s="3">
+        <f t="shared" si="0"/>
+        <v>2303836</v>
+      </c>
+      <c r="F16" s="3">
+        <f t="shared" si="1"/>
+        <v>-58980</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
         <v>45931</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="3">
         <v>2418070</v>
       </c>
-      <c r="C17">
-        <f t="shared" si="0"/>
-        <v>2643262</v>
-      </c>
-      <c r="D17">
-        <v>-225192</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C17" s="3">
+        <v>699111</v>
+      </c>
+      <c r="D17" s="3">
+        <v>1910607</v>
+      </c>
+      <c r="E17" s="3">
+        <f t="shared" si="0"/>
+        <v>2609718</v>
+      </c>
+      <c r="F17" s="3">
+        <f t="shared" si="1"/>
+        <v>-191648</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
         <v>45962</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="3">
         <v>1972220</v>
       </c>
-      <c r="C18">
-        <f t="shared" si="0"/>
-        <v>2138672</v>
-      </c>
-      <c r="D18">
-        <v>-166452</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C18" s="3">
+        <v>600645</v>
+      </c>
+      <c r="D18" s="3">
+        <v>1487729</v>
+      </c>
+      <c r="E18" s="3">
+        <f t="shared" si="0"/>
+        <v>2088374</v>
+      </c>
+      <c r="F18" s="3">
+        <f t="shared" si="1"/>
+        <v>-116154</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
         <v>45992</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="3">
         <v>2411809</v>
       </c>
-      <c r="C19">
-        <f t="shared" si="0"/>
-        <v>2235684</v>
-      </c>
-      <c r="D19">
-        <v>176125</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C19" s="3">
+        <v>672021</v>
+      </c>
+      <c r="D19" s="3">
+        <v>1544402</v>
+      </c>
+      <c r="E19" s="3">
+        <f t="shared" si="0"/>
+        <v>2216423</v>
+      </c>
+      <c r="F19" s="3">
+        <f t="shared" si="1"/>
+        <v>195386</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
         <v>46023</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="3">
         <v>1686045</v>
       </c>
-      <c r="C20">
-        <f t="shared" si="0"/>
-        <v>1557016</v>
-      </c>
-      <c r="D20">
-        <v>129029</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C20" s="3">
+        <v>7549</v>
+      </c>
+      <c r="D20" s="3">
+        <v>1601282</v>
+      </c>
+      <c r="E20" s="3">
+        <f t="shared" si="0"/>
+        <v>1608831</v>
+      </c>
+      <c r="F20" s="3">
+        <f t="shared" si="1"/>
+        <v>77214</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
         <v>46054</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="3">
         <v>1646609</v>
       </c>
-      <c r="C21">
-        <f t="shared" si="0"/>
-        <v>1614992</v>
-      </c>
-      <c r="D21">
-        <v>31617</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C21" s="3">
+        <v>16213</v>
+      </c>
+      <c r="D21" s="3">
+        <v>1568310</v>
+      </c>
+      <c r="E21" s="3">
+        <f t="shared" si="0"/>
+        <v>1584523</v>
+      </c>
+      <c r="F21" s="3">
+        <f t="shared" si="1"/>
+        <v>62086</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
         <v>46082</v>
       </c>
-      <c r="B22">
+      <c r="B22" s="3">
         <v>1861769</v>
       </c>
-      <c r="C22">
-        <f t="shared" si="0"/>
-        <v>1674430</v>
-      </c>
-      <c r="D22">
-        <v>187339</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C22" s="3">
+        <v>22825</v>
+      </c>
+      <c r="D22" s="3">
+        <v>1711521</v>
+      </c>
+      <c r="E22" s="3">
+        <f t="shared" si="0"/>
+        <v>1734346</v>
+      </c>
+      <c r="F22" s="3">
+        <f t="shared" si="1"/>
+        <v>127423</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
         <v>46113</v>
       </c>
-      <c r="B23">
+      <c r="B23" s="3">
         <v>2062624</v>
       </c>
-      <c r="C23">
-        <f t="shared" si="0"/>
-        <v>1997175</v>
-      </c>
-      <c r="D23">
-        <v>65449</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C23" s="3">
+        <v>51423</v>
+      </c>
+      <c r="D23" s="3">
+        <v>1920333</v>
+      </c>
+      <c r="E23" s="3">
+        <f t="shared" si="0"/>
+        <v>1971756</v>
+      </c>
+      <c r="F23" s="3">
+        <f t="shared" si="1"/>
+        <v>90868</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
         <v>46143</v>
       </c>
-      <c r="B24">
+      <c r="B24" s="3">
         <v>2028185</v>
       </c>
-      <c r="C24">
-        <f t="shared" si="0"/>
-        <v>1861458</v>
-      </c>
-      <c r="D24">
-        <v>166727</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C24" s="3">
+        <v>67926</v>
+      </c>
+      <c r="D24" s="3">
+        <v>1762572</v>
+      </c>
+      <c r="E24" s="3">
+        <f t="shared" si="0"/>
+        <v>1830498</v>
+      </c>
+      <c r="F24" s="3">
+        <f t="shared" si="1"/>
+        <v>197687</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
         <v>46174</v>
       </c>
-      <c r="B25">
+      <c r="B25" s="3">
         <v>2099555</v>
       </c>
-      <c r="C25">
-        <f t="shared" si="0"/>
-        <v>1918430</v>
-      </c>
-      <c r="D25">
-        <v>181125</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C25" s="3">
+        <v>79119</v>
+      </c>
+      <c r="D25" s="3">
+        <v>1812796</v>
+      </c>
+      <c r="E25" s="3">
+        <f t="shared" si="0"/>
+        <v>1891915</v>
+      </c>
+      <c r="F25" s="3">
+        <f t="shared" si="1"/>
+        <v>207640</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
         <v>46204</v>
+      </c>
+      <c r="B26" s="3">
+        <v>2443965</v>
+      </c>
+      <c r="C26" s="3">
+        <v>73004</v>
+      </c>
+      <c r="D26" s="3">
+        <v>1708237</v>
+      </c>
+      <c r="E26" s="3">
+        <f t="shared" si="0"/>
+        <v>1781241</v>
+      </c>
+      <c r="F26" s="3">
+        <f t="shared" si="1"/>
+        <v>662724</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Explain Home COGS drop as a Casey/Nate accounting reclassification
Through Dec 2025 the books credited Casey for raw milk production and
debited Nate for the milk cost as an offsetting wash entry, inflating
both Revenue and COGS equally; that stopped Jan 2026. Restate the
Home revenue/costs chart and Financials table onto one consistent
basis (trailing 12 months before Jul 1, 2026) using the workbook's
new "adj" sheet, and note the reclassification as a footnote on the
executive summary rather than treating the COGS drop as unexplained.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Monthly Revenue vs. Operating Costs.xlsx
+++ b/data/Monthly Revenue vs. Operating Costs.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oliviaarkema/Documents/Strategic Planning/CD_StrategicPlanning/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC83C91C-6B59-C848-9493-64C92FABA782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78C05C6C-6583-8747-ACB2-ACCB1E04CBAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="-5700" windowWidth="38400" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
+    <sheet name="adj" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="7">
   <si>
     <t>Month</t>
   </si>
@@ -52,6 +53,9 @@
   <si>
     <t>Net Ordinary Income (Not Including Other Income &amp; Expenses)</t>
   </si>
+  <si>
+    <t>ADJ</t>
+  </si>
 </sst>
 </file>
 
@@ -59,7 +63,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -104,11 +108,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -446,7 +451,7 @@
         <v>45474</v>
       </c>
       <c r="B2" s="3">
-        <v>2349438</v>
+        <v>1607862</v>
       </c>
       <c r="C2" s="3">
         <v>741576</v>
@@ -455,8 +460,8 @@
         <v>1373637</v>
       </c>
       <c r="E2" s="3">
-        <f>C2+D2</f>
-        <v>2115213</v>
+        <f>D2</f>
+        <v>1373637</v>
       </c>
       <c r="F2" s="3">
         <f>B2-E2</f>
@@ -468,7 +473,7 @@
         <v>45505</v>
       </c>
       <c r="B3" s="3">
-        <v>2299610</v>
+        <v>1606221</v>
       </c>
       <c r="C3" s="3">
         <v>693389</v>
@@ -477,8 +482,8 @@
         <v>1620287</v>
       </c>
       <c r="E3" s="3">
-        <f t="shared" ref="E3:E26" si="0">C3+D3</f>
-        <v>2313676</v>
+        <f t="shared" ref="E3:E19" si="0">D3</f>
+        <v>1620287</v>
       </c>
       <c r="F3" s="3">
         <f t="shared" ref="F3:F26" si="1">B3-E3</f>
@@ -490,7 +495,7 @@
         <v>45536</v>
       </c>
       <c r="B4" s="3">
-        <v>2055377</v>
+        <v>1395122</v>
       </c>
       <c r="C4" s="3">
         <v>660255</v>
@@ -500,7 +505,7 @@
       </c>
       <c r="E4" s="3">
         <f t="shared" si="0"/>
-        <v>2108503</v>
+        <v>1448248</v>
       </c>
       <c r="F4" s="3">
         <f t="shared" si="1"/>
@@ -512,7 +517,7 @@
         <v>45566</v>
       </c>
       <c r="B5" s="3">
-        <v>2225430</v>
+        <v>1555498</v>
       </c>
       <c r="C5" s="3">
         <v>669932</v>
@@ -522,7 +527,7 @@
       </c>
       <c r="E5" s="3">
         <f t="shared" si="0"/>
-        <v>2038955</v>
+        <v>1369023</v>
       </c>
       <c r="F5" s="3">
         <f t="shared" si="1"/>
@@ -534,7 +539,7 @@
         <v>45597</v>
       </c>
       <c r="B6" s="3">
-        <v>2138141</v>
+        <v>1505900</v>
       </c>
       <c r="C6" s="3">
         <v>632241</v>
@@ -544,7 +549,7 @@
       </c>
       <c r="E6" s="3">
         <f t="shared" si="0"/>
-        <v>2093132</v>
+        <v>1460891</v>
       </c>
       <c r="F6" s="3">
         <f t="shared" si="1"/>
@@ -556,7 +561,7 @@
         <v>45627</v>
       </c>
       <c r="B7" s="3">
-        <v>2086631</v>
+        <v>1443558</v>
       </c>
       <c r="C7" s="3">
         <v>643073</v>
@@ -566,7 +571,7 @@
       </c>
       <c r="E7" s="3">
         <f t="shared" si="0"/>
-        <v>2144030</v>
+        <v>1500957</v>
       </c>
       <c r="F7" s="3">
         <f t="shared" si="1"/>
@@ -578,7 +583,7 @@
         <v>45658</v>
       </c>
       <c r="B8" s="3">
-        <v>2079507</v>
+        <v>1412950</v>
       </c>
       <c r="C8" s="3">
         <v>666557</v>
@@ -588,7 +593,7 @@
       </c>
       <c r="E8" s="3">
         <f t="shared" si="0"/>
-        <v>2199971</v>
+        <v>1533414</v>
       </c>
       <c r="F8" s="3">
         <f t="shared" si="1"/>
@@ -600,7 +605,7 @@
         <v>45689</v>
       </c>
       <c r="B9" s="3">
-        <v>1772753</v>
+        <v>1243821</v>
       </c>
       <c r="C9" s="3">
         <v>528932</v>
@@ -610,7 +615,7 @@
       </c>
       <c r="E9" s="3">
         <f t="shared" si="0"/>
-        <v>1808808</v>
+        <v>1279876</v>
       </c>
       <c r="F9" s="3">
         <f t="shared" si="1"/>
@@ -622,7 +627,7 @@
         <v>45717</v>
       </c>
       <c r="B10" s="3">
-        <v>2087068</v>
+        <v>1480489</v>
       </c>
       <c r="C10" s="3">
         <v>606579</v>
@@ -632,7 +637,7 @@
       </c>
       <c r="E10" s="3">
         <f t="shared" si="0"/>
-        <v>2012894</v>
+        <v>1406315</v>
       </c>
       <c r="F10" s="3">
         <f t="shared" si="1"/>
@@ -644,7 +649,7 @@
         <v>45748</v>
       </c>
       <c r="B11" s="3">
-        <v>2184308</v>
+        <v>1583975</v>
       </c>
       <c r="C11" s="3">
         <v>600333</v>
@@ -654,7 +659,7 @@
       </c>
       <c r="E11" s="3">
         <f t="shared" si="0"/>
-        <v>2178820</v>
+        <v>1578487</v>
       </c>
       <c r="F11" s="3">
         <f t="shared" si="1"/>
@@ -666,7 +671,7 @@
         <v>45778</v>
       </c>
       <c r="B12" s="3">
-        <v>2277922</v>
+        <v>1629215</v>
       </c>
       <c r="C12" s="3">
         <v>648707</v>
@@ -676,7 +681,7 @@
       </c>
       <c r="E12" s="3">
         <f t="shared" si="0"/>
-        <v>2211062</v>
+        <v>1562355</v>
       </c>
       <c r="F12" s="3">
         <f t="shared" si="1"/>
@@ -688,7 +693,7 @@
         <v>45809</v>
       </c>
       <c r="B13" s="3">
-        <v>2523351</v>
+        <v>1788412</v>
       </c>
       <c r="C13" s="3">
         <v>734939</v>
@@ -698,7 +703,7 @@
       </c>
       <c r="E13" s="3">
         <f t="shared" si="0"/>
-        <v>2431456</v>
+        <v>1696517</v>
       </c>
       <c r="F13" s="3">
         <f t="shared" si="1"/>
@@ -710,7 +715,7 @@
         <v>45839</v>
       </c>
       <c r="B14" s="3">
-        <v>2585013</v>
+        <v>1894218</v>
       </c>
       <c r="C14" s="3">
         <v>690795</v>
@@ -720,7 +725,7 @@
       </c>
       <c r="E14" s="3">
         <f t="shared" si="0"/>
-        <v>2585382</v>
+        <v>1894587</v>
       </c>
       <c r="F14" s="3">
         <f t="shared" si="1"/>
@@ -732,7 +737,7 @@
         <v>45870</v>
       </c>
       <c r="B15" s="3">
-        <v>2466680</v>
+        <v>1718749</v>
       </c>
       <c r="C15" s="3">
         <v>747931</v>
@@ -742,7 +747,7 @@
       </c>
       <c r="E15" s="3">
         <f t="shared" si="0"/>
-        <v>2303469</v>
+        <v>1555538</v>
       </c>
       <c r="F15" s="3">
         <f t="shared" si="1"/>
@@ -754,7 +759,7 @@
         <v>45901</v>
       </c>
       <c r="B16" s="3">
-        <v>2244856</v>
+        <v>1558587</v>
       </c>
       <c r="C16" s="3">
         <v>686269</v>
@@ -764,7 +769,7 @@
       </c>
       <c r="E16" s="3">
         <f t="shared" si="0"/>
-        <v>2303836</v>
+        <v>1617567</v>
       </c>
       <c r="F16" s="3">
         <f t="shared" si="1"/>
@@ -776,7 +781,7 @@
         <v>45931</v>
       </c>
       <c r="B17" s="3">
-        <v>2418070</v>
+        <v>1718959</v>
       </c>
       <c r="C17" s="3">
         <v>699111</v>
@@ -786,7 +791,7 @@
       </c>
       <c r="E17" s="3">
         <f t="shared" si="0"/>
-        <v>2609718</v>
+        <v>1910607</v>
       </c>
       <c r="F17" s="3">
         <f t="shared" si="1"/>
@@ -798,7 +803,7 @@
         <v>45962</v>
       </c>
       <c r="B18" s="3">
-        <v>1972220</v>
+        <v>1371575</v>
       </c>
       <c r="C18" s="3">
         <v>600645</v>
@@ -808,7 +813,7 @@
       </c>
       <c r="E18" s="3">
         <f t="shared" si="0"/>
-        <v>2088374</v>
+        <v>1487729</v>
       </c>
       <c r="F18" s="3">
         <f t="shared" si="1"/>
@@ -820,7 +825,7 @@
         <v>45992</v>
       </c>
       <c r="B19" s="3">
-        <v>2411809</v>
+        <v>1739788</v>
       </c>
       <c r="C19" s="3">
         <v>672021</v>
@@ -830,7 +835,7 @@
       </c>
       <c r="E19" s="3">
         <f t="shared" si="0"/>
-        <v>2216423</v>
+        <v>1544402</v>
       </c>
       <c r="F19" s="3">
         <f t="shared" si="1"/>
@@ -851,7 +856,7 @@
         <v>1601282</v>
       </c>
       <c r="E20" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="E3:E26" si="2">C20+D20</f>
         <v>1608831</v>
       </c>
       <c r="F20" s="3">
@@ -873,7 +878,7 @@
         <v>1568310</v>
       </c>
       <c r="E21" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1584523</v>
       </c>
       <c r="F21" s="3">
@@ -895,7 +900,7 @@
         <v>1711521</v>
       </c>
       <c r="E22" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1734346</v>
       </c>
       <c r="F22" s="3">
@@ -917,7 +922,7 @@
         <v>1920333</v>
       </c>
       <c r="E23" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1971756</v>
       </c>
       <c r="F23" s="3">
@@ -939,7 +944,7 @@
         <v>1762572</v>
       </c>
       <c r="E24" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1830498</v>
       </c>
       <c r="F24" s="3">
@@ -961,7 +966,7 @@
         <v>1812796</v>
       </c>
       <c r="E25" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1891915</v>
       </c>
       <c r="F25" s="3">
@@ -983,7 +988,7 @@
         <v>1708237</v>
       </c>
       <c r="E26" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1781241</v>
       </c>
       <c r="F26" s="3">
@@ -994,4 +999,301 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D58A040-9CF5-5C41-87AE-A21F32AFB144}">
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="4" max="4" width="11.1640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" s="2">
+        <v>45474</v>
+      </c>
+      <c r="B2" s="3">
+        <v>2349438</v>
+      </c>
+      <c r="C2" s="3">
+        <v>741576</v>
+      </c>
+      <c r="D2" s="4">
+        <f>B2-C2</f>
+        <v>1607862</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" s="2">
+        <v>45505</v>
+      </c>
+      <c r="B3" s="3">
+        <v>2299610</v>
+      </c>
+      <c r="C3" s="3">
+        <v>693389</v>
+      </c>
+      <c r="D3" s="4">
+        <f t="shared" ref="D3:D19" si="0">B3-C3</f>
+        <v>1606221</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="2">
+        <v>45536</v>
+      </c>
+      <c r="B4" s="3">
+        <v>2055377</v>
+      </c>
+      <c r="C4" s="3">
+        <v>660255</v>
+      </c>
+      <c r="D4" s="4">
+        <f t="shared" si="0"/>
+        <v>1395122</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="2">
+        <v>45566</v>
+      </c>
+      <c r="B5" s="3">
+        <v>2225430</v>
+      </c>
+      <c r="C5" s="3">
+        <v>669932</v>
+      </c>
+      <c r="D5" s="4">
+        <f t="shared" si="0"/>
+        <v>1555498</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="2">
+        <v>45597</v>
+      </c>
+      <c r="B6" s="3">
+        <v>2138141</v>
+      </c>
+      <c r="C6" s="3">
+        <v>632241</v>
+      </c>
+      <c r="D6" s="4">
+        <f t="shared" si="0"/>
+        <v>1505900</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" s="2">
+        <v>45627</v>
+      </c>
+      <c r="B7" s="3">
+        <v>2086631</v>
+      </c>
+      <c r="C7" s="3">
+        <v>643073</v>
+      </c>
+      <c r="D7" s="4">
+        <f t="shared" si="0"/>
+        <v>1443558</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="2">
+        <v>45658</v>
+      </c>
+      <c r="B8" s="3">
+        <v>2079507</v>
+      </c>
+      <c r="C8" s="3">
+        <v>666557</v>
+      </c>
+      <c r="D8" s="4">
+        <f t="shared" si="0"/>
+        <v>1412950</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" s="2">
+        <v>45689</v>
+      </c>
+      <c r="B9" s="3">
+        <v>1772753</v>
+      </c>
+      <c r="C9" s="3">
+        <v>528932</v>
+      </c>
+      <c r="D9" s="4">
+        <f t="shared" si="0"/>
+        <v>1243821</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" s="2">
+        <v>45717</v>
+      </c>
+      <c r="B10" s="3">
+        <v>2087068</v>
+      </c>
+      <c r="C10" s="3">
+        <v>606579</v>
+      </c>
+      <c r="D10" s="4">
+        <f t="shared" si="0"/>
+        <v>1480489</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" s="2">
+        <v>45748</v>
+      </c>
+      <c r="B11" s="3">
+        <v>2184308</v>
+      </c>
+      <c r="C11" s="3">
+        <v>600333</v>
+      </c>
+      <c r="D11" s="4">
+        <f t="shared" si="0"/>
+        <v>1583975</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" s="2">
+        <v>45778</v>
+      </c>
+      <c r="B12" s="3">
+        <v>2277922</v>
+      </c>
+      <c r="C12" s="3">
+        <v>648707</v>
+      </c>
+      <c r="D12" s="4">
+        <f t="shared" si="0"/>
+        <v>1629215</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" s="2">
+        <v>45809</v>
+      </c>
+      <c r="B13" s="3">
+        <v>2523351</v>
+      </c>
+      <c r="C13" s="3">
+        <v>734939</v>
+      </c>
+      <c r="D13" s="4">
+        <f t="shared" si="0"/>
+        <v>1788412</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" s="2">
+        <v>45839</v>
+      </c>
+      <c r="B14" s="3">
+        <v>2585013</v>
+      </c>
+      <c r="C14" s="3">
+        <v>690795</v>
+      </c>
+      <c r="D14" s="4">
+        <f t="shared" si="0"/>
+        <v>1894218</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" s="2">
+        <v>45870</v>
+      </c>
+      <c r="B15" s="3">
+        <v>2466680</v>
+      </c>
+      <c r="C15" s="3">
+        <v>747931</v>
+      </c>
+      <c r="D15" s="4">
+        <f t="shared" si="0"/>
+        <v>1718749</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" s="2">
+        <v>45901</v>
+      </c>
+      <c r="B16" s="3">
+        <v>2244856</v>
+      </c>
+      <c r="C16" s="3">
+        <v>686269</v>
+      </c>
+      <c r="D16" s="4">
+        <f t="shared" si="0"/>
+        <v>1558587</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" s="2">
+        <v>45931</v>
+      </c>
+      <c r="B17" s="3">
+        <v>2418070</v>
+      </c>
+      <c r="C17" s="3">
+        <v>699111</v>
+      </c>
+      <c r="D17" s="4">
+        <f t="shared" si="0"/>
+        <v>1718959</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" s="2">
+        <v>45962</v>
+      </c>
+      <c r="B18" s="3">
+        <v>1972220</v>
+      </c>
+      <c r="C18" s="3">
+        <v>600645</v>
+      </c>
+      <c r="D18" s="4">
+        <f t="shared" si="0"/>
+        <v>1371575</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" s="2">
+        <v>45992</v>
+      </c>
+      <c r="B19" s="3">
+        <v>2411809</v>
+      </c>
+      <c r="C19" s="3">
+        <v>672021</v>
+      </c>
+      <c r="D19" s="4">
+        <f t="shared" si="0"/>
+        <v>1739788</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>